<commit_message>
ml: update the sch sth forms
</commit_message>
<xml_diff>
--- a/SCH-STH/Impact assessments/Mali/2025/ml_sch_sth_impact_2501_1_school.xlsx
+++ b/SCH-STH/Impact assessments/Mali/2025/ml_sch_sth_impact_2501_1_school.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\SCH-STH\Impact assessments\Mali\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2076FFB5-65DC-496C-8D88-6AD7102D1EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624A8E09-DE0D-4F77-9646-5F6D9F1AE8D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2680" uniqueCount="663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2682" uniqueCount="664">
   <si>
     <t>type</t>
   </si>
@@ -2209,6 +2209,9 @@
   </si>
   <si>
     <t>allow_choice_duplicates</t>
+  </si>
+  <si>
+    <t>${w_subdistrict_1} != 'Autre'</t>
   </si>
 </sst>
 </file>
@@ -3065,7 +3068,7 @@
       <c r="O7" s="33"/>
       <c r="P7" s="33"/>
     </row>
-    <row r="8" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" s="5" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
@@ -3079,7 +3082,9 @@
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
       <c r="G8" s="10"/>
-      <c r="H8" s="9"/>
+      <c r="H8" s="9" t="s">
+        <v>663</v>
+      </c>
       <c r="I8" s="9"/>
       <c r="J8" s="9" t="s">
         <v>12</v>
@@ -3169,7 +3174,9 @@
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
       <c r="G11" s="10"/>
-      <c r="H11" s="9"/>
+      <c r="H11" s="9" t="s">
+        <v>663</v>
+      </c>
       <c r="I11" s="9"/>
       <c r="J11" s="9" t="s">
         <v>12</v>

</xml_diff>